<commit_message>
commit before pilot_23: replace broom concept with knife
</commit_message>
<xml_diff>
--- a/psychopy_exp_files/sequences/localizer_conditions_things-meg_mixed_5cat_04.xlsx
+++ b/psychopy_exp_files/sequences/localizer_conditions_things-meg_mixed_5cat_04.xlsx
@@ -606,7 +606,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -620,17 +620,17 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_01.png</t>
+          <t>boat\boat_01.png</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -935,7 +935,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M8" t="n">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G14" t="n">
@@ -1299,17 +1299,17 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>broom\broom_05.png</t>
+          <t>knife\knife_05.png</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M14" t="n">
@@ -1407,7 +1407,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G16" t="n">
@@ -1421,17 +1421,17 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_12.png</t>
+          <t>boat\boat_12.png</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M16" t="n">
@@ -1590,7 +1590,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G19" t="n">
@@ -1604,17 +1604,17 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>broom\broom_08.png</t>
+          <t>knife\knife_08.png</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M19" t="n">
@@ -1651,7 +1651,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G20" t="n">
@@ -1665,17 +1665,17 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_09.png</t>
+          <t>boat\boat_09.png</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M20" t="n">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G21" t="n">
@@ -1726,7 +1726,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>broom\broom_04.png</t>
+          <t>knife\knife_04.png</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -2094,7 +2094,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G27" t="n">
@@ -2108,17 +2108,17 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_10.png</t>
+          <t>boat\boat_10.png</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M27" t="n">
@@ -2179,7 +2179,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M28" t="n">
@@ -2301,7 +2301,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M30" t="n">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M35" t="n">
@@ -2651,7 +2651,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G36" t="n">
@@ -2665,17 +2665,17 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>broom\broom_03.png</t>
+          <t>knife\knife_03.png</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M36" t="n">
@@ -2834,7 +2834,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G39" t="n">
@@ -2848,17 +2848,17 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_04.png</t>
+          <t>boat\boat_04.png</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M39" t="n">
@@ -3102,7 +3102,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M43" t="n">
@@ -3232,7 +3232,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M45" t="n">
@@ -3537,7 +3537,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M50" t="n">
@@ -3635,7 +3635,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G52" t="n">
@@ -3649,17 +3649,17 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>broom\broom_12.png</t>
+          <t>knife\knife_12.png</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M52" t="n">
@@ -3757,7 +3757,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G54" t="n">
@@ -3771,17 +3771,17 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>broom\broom_07.png</t>
+          <t>knife\knife_07.png</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M54" t="n">
@@ -3879,7 +3879,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G56" t="n">
@@ -3893,17 +3893,17 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_02.png</t>
+          <t>boat\boat_02.png</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M56" t="n">
@@ -4131,7 +4131,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G60" t="n">
@@ -4145,17 +4145,17 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_11.png</t>
+          <t>boat\boat_11.png</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M60" t="n">
@@ -4253,7 +4253,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G62" t="n">
@@ -4267,17 +4267,17 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>broom\broom_02.png</t>
+          <t>knife\knife_02.png</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M62" t="n">
@@ -4619,7 +4619,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G68" t="n">
@@ -4633,7 +4633,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_03.png</t>
+          <t>boat\boat_03.png</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4993,7 +4993,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G74" t="n">
@@ -5007,17 +5007,17 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>broom\broom_10.png</t>
+          <t>knife\knife_10.png</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M74" t="n">
@@ -5115,7 +5115,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G76" t="n">
@@ -5129,17 +5129,17 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_06.png</t>
+          <t>boat\boat_06.png</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M76" t="n">
@@ -5513,7 +5513,7 @@
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M82" t="n">
@@ -5757,7 +5757,7 @@
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M86" t="n">
@@ -5813,12 +5813,12 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M87" t="n">
@@ -6192,7 +6192,7 @@
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M93" t="n">
@@ -6229,7 +6229,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G94" t="n">
@@ -6243,17 +6243,17 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_05.png</t>
+          <t>boat\boat_05.png</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L94" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M94" t="n">
@@ -6436,7 +6436,7 @@
       </c>
       <c r="L97" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M97" t="n">
@@ -6566,7 +6566,7 @@
       </c>
       <c r="L99" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M99" t="n">
@@ -6725,7 +6725,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G102" t="n">
@@ -6739,17 +6739,17 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>broom\broom_09.png</t>
+          <t>knife\knife_09.png</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L102" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M102" t="n">
@@ -6810,7 +6810,7 @@
       </c>
       <c r="L103" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M103" t="n">
@@ -6847,7 +6847,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G104" t="n">
@@ -6861,17 +6861,17 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>broom\broom_04.png</t>
+          <t>knife\knife_04.png</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L104" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M104" t="n">
@@ -7160,7 +7160,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G109" t="n">
@@ -7174,17 +7174,17 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_10.png</t>
+          <t>boat\boat_10.png</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M109" t="n">
@@ -7282,7 +7282,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G111" t="n">
@@ -7296,17 +7296,17 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>broom\broom_06.png</t>
+          <t>knife\knife_06.png</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L111" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M111" t="n">
@@ -7595,7 +7595,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G116" t="n">
@@ -7609,17 +7609,17 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>broom\broom_01.png</t>
+          <t>knife\knife_01.png</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L116" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M116" t="n">
@@ -7778,7 +7778,7 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G119" t="n">
@@ -7792,17 +7792,17 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_13.png</t>
+          <t>boat\boat_13.png</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L119" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M119" t="n">
@@ -7863,7 +7863,7 @@
       </c>
       <c r="L120" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M120" t="n">
@@ -8335,7 +8335,7 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G128" t="n">
@@ -8349,17 +8349,17 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>broom\broom_11.png</t>
+          <t>knife\knife_11.png</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L128" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M128" t="n">
@@ -8420,7 +8420,7 @@
       </c>
       <c r="L129" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M129" t="n">
@@ -8579,7 +8579,7 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G132" t="n">
@@ -8593,7 +8593,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_07.png</t>
+          <t>boat\boat_07.png</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8855,7 +8855,7 @@
       </c>
       <c r="L136" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M136" t="n">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G139" t="n">
@@ -9028,17 +9028,17 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_05.png</t>
+          <t>boat\boat_05.png</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L139" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M139" t="n">
@@ -9282,7 +9282,7 @@
       </c>
       <c r="L143" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M143" t="n">
@@ -9441,7 +9441,7 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G146" t="n">
@@ -9455,17 +9455,17 @@
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_08.png</t>
+          <t>boat\boat_08.png</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L146" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M146" t="n">
@@ -9582,12 +9582,12 @@
       </c>
       <c r="K148" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L148" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M148" t="n">
@@ -9815,7 +9815,7 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G152" t="n">
@@ -9829,17 +9829,17 @@
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>broom\broom_02.png</t>
+          <t>knife\knife_02.png</t>
         </is>
       </c>
       <c r="K152" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L152" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M152" t="n">
@@ -9876,7 +9876,7 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G153" t="n">
@@ -9890,17 +9890,17 @@
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_11.png</t>
+          <t>boat\boat_11.png</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L153" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M153" t="n">
@@ -9937,7 +9937,7 @@
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G154" t="n">
@@ -9951,17 +9951,17 @@
       </c>
       <c r="J154" t="inlineStr">
         <is>
-          <t>broom\broom_03.png</t>
+          <t>knife\knife_03.png</t>
         </is>
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L154" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M154" t="n">
@@ -10616,7 +10616,7 @@
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G165" t="n">
@@ -10630,17 +10630,17 @@
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_04.png</t>
+          <t>boat\boat_04.png</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L165" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M165" t="n">
@@ -10818,12 +10818,12 @@
       </c>
       <c r="K168" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L168" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M168" t="n">
@@ -10929,7 +10929,7 @@
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G170" t="n">
@@ -10943,17 +10943,17 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>broom\broom_01.png</t>
+          <t>knife\knife_01.png</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L170" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M170" t="n">
@@ -11075,7 +11075,7 @@
       </c>
       <c r="L172" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M172" t="n">
@@ -11112,7 +11112,7 @@
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G173" t="n">
@@ -11126,17 +11126,17 @@
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_07.png</t>
+          <t>boat\boat_07.png</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L173" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M173" t="n">
@@ -11441,7 +11441,7 @@
       </c>
       <c r="L178" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M178" t="n">
@@ -11547,7 +11547,7 @@
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G180" t="n">
@@ -11561,17 +11561,17 @@
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>broom\broom_08.png</t>
+          <t>knife\knife_08.png</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L180" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M180" t="n">
@@ -11754,7 +11754,7 @@
       </c>
       <c r="L183" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M183" t="n">
@@ -12096,7 +12096,7 @@
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G189" t="n">
@@ -12110,7 +12110,7 @@
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_12.png</t>
+          <t>boat\boat_12.png</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -12189,7 +12189,7 @@
       </c>
       <c r="L190" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M190" t="n">
@@ -12348,7 +12348,7 @@
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G193" t="n">
@@ -12362,17 +12362,17 @@
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_08.png</t>
+          <t>boat\boat_08.png</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L193" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M193" t="n">
@@ -12494,7 +12494,7 @@
       </c>
       <c r="L195" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M195" t="n">
@@ -12616,7 +12616,7 @@
       </c>
       <c r="L197" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M197" t="n">
@@ -12775,7 +12775,7 @@
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G200" t="n">
@@ -12789,7 +12789,7 @@
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>broom\broom_07.png</t>
+          <t>knife\knife_07.png</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
@@ -13157,7 +13157,7 @@
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G206" t="n">
@@ -13171,17 +13171,17 @@
       </c>
       <c r="J206" t="inlineStr">
         <is>
-          <t>broom\broom_12.png</t>
+          <t>knife\knife_12.png</t>
         </is>
       </c>
       <c r="K206" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L206" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M206" t="n">
@@ -13279,7 +13279,7 @@
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G208" t="n">
@@ -13293,17 +13293,17 @@
       </c>
       <c r="J208" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_09.png</t>
+          <t>boat\boat_09.png</t>
         </is>
       </c>
       <c r="K208" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L208" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M208" t="n">
@@ -13462,7 +13462,7 @@
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G211" t="n">
@@ -13476,17 +13476,17 @@
       </c>
       <c r="J211" t="inlineStr">
         <is>
-          <t>broom\broom_06.png</t>
+          <t>knife\knife_06.png</t>
         </is>
       </c>
       <c r="K211" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L211" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M211" t="n">
@@ -13664,12 +13664,12 @@
       </c>
       <c r="K214" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L214" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M214" t="n">
@@ -13799,7 +13799,7 @@
       </c>
       <c r="L216" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M216" t="n">
@@ -14019,7 +14019,7 @@
       </c>
       <c r="F220" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G220" t="n">
@@ -14033,17 +14033,17 @@
       </c>
       <c r="J220" t="inlineStr">
         <is>
-          <t>broom\broom_11.png</t>
+          <t>knife\knife_11.png</t>
         </is>
       </c>
       <c r="K220" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L220" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M220" t="n">
@@ -14141,7 +14141,7 @@
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G222" t="n">
@@ -14155,17 +14155,17 @@
       </c>
       <c r="J222" t="inlineStr">
         <is>
-          <t>broom\broom_10.png</t>
+          <t>knife\knife_10.png</t>
         </is>
       </c>
       <c r="K222" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L222" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M222" t="n">
@@ -14226,7 +14226,7 @@
       </c>
       <c r="L223" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M223" t="n">
@@ -14515,7 +14515,7 @@
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G228" t="n">
@@ -14529,17 +14529,17 @@
       </c>
       <c r="J228" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_13.png</t>
+          <t>boat\boat_13.png</t>
         </is>
       </c>
       <c r="K228" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L228" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M228" t="n">
@@ -14844,7 +14844,7 @@
       </c>
       <c r="L233" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M233" t="n">
@@ -14974,7 +14974,7 @@
       </c>
       <c r="L235" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M235" t="n">
@@ -15011,7 +15011,7 @@
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G236" t="n">
@@ -15025,17 +15025,17 @@
       </c>
       <c r="J236" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_01.png</t>
+          <t>boat\boat_01.png</t>
         </is>
       </c>
       <c r="K236" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L236" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M236" t="n">
@@ -15377,7 +15377,7 @@
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G242" t="n">
@@ -15391,17 +15391,17 @@
       </c>
       <c r="J242" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_02.png</t>
+          <t>boat\boat_02.png</t>
         </is>
       </c>
       <c r="K242" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L242" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M242" t="n">
@@ -15462,7 +15462,7 @@
       </c>
       <c r="L243" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M243" t="n">
@@ -15560,7 +15560,7 @@
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G245" t="n">
@@ -15574,17 +15574,17 @@
       </c>
       <c r="J245" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_06.png</t>
+          <t>boat\boat_06.png</t>
         </is>
       </c>
       <c r="K245" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L245" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M245" t="n">
@@ -15836,7 +15836,7 @@
       </c>
       <c r="L249" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M249" t="n">
@@ -15958,7 +15958,7 @@
       </c>
       <c r="L251" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M251" t="n">
@@ -16056,7 +16056,7 @@
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G253" t="n">
@@ -16070,17 +16070,17 @@
       </c>
       <c r="J253" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_09.png</t>
+          <t>boat\boat_09.png</t>
         </is>
       </c>
       <c r="K253" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L253" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M253" t="n">
@@ -16247,7 +16247,7 @@
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G256" t="n">
@@ -16261,17 +16261,17 @@
       </c>
       <c r="J256" t="inlineStr">
         <is>
-          <t>broom\broom_03.png</t>
+          <t>knife\knife_03.png</t>
         </is>
       </c>
       <c r="K256" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L256" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M256" t="n">
@@ -16369,7 +16369,7 @@
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G258" t="n">
@@ -16383,17 +16383,17 @@
       </c>
       <c r="J258" t="inlineStr">
         <is>
-          <t>broom\broom_09.png</t>
+          <t>knife\knife_09.png</t>
         </is>
       </c>
       <c r="K258" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L258" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M258" t="n">
@@ -16552,7 +16552,7 @@
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G261" t="n">
@@ -16566,17 +16566,17 @@
       </c>
       <c r="J261" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_12.png</t>
+          <t>boat\boat_12.png</t>
         </is>
       </c>
       <c r="K261" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L261" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M261" t="n">
@@ -16613,7 +16613,7 @@
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G262" t="n">
@@ -16627,17 +16627,17 @@
       </c>
       <c r="J262" t="inlineStr">
         <is>
-          <t>broom\broom_05.png</t>
+          <t>knife\knife_05.png</t>
         </is>
       </c>
       <c r="K262" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L262" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M262" t="n">
@@ -16759,7 +16759,7 @@
       </c>
       <c r="L264" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M264" t="n">
@@ -16876,12 +16876,12 @@
       </c>
       <c r="K266" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L266" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M266" t="n">
@@ -16926,7 +16926,7 @@
       </c>
       <c r="F267" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G267" t="n">
@@ -16940,17 +16940,17 @@
       </c>
       <c r="J267" t="inlineStr">
         <is>
-          <t>broom\broom_10.png</t>
+          <t>knife\knife_10.png</t>
         </is>
       </c>
       <c r="K267" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L267" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M267" t="n">
@@ -16987,7 +16987,7 @@
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G268" t="n">
@@ -17001,17 +17001,17 @@
       </c>
       <c r="J268" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_04.png</t>
+          <t>boat\boat_04.png</t>
         </is>
       </c>
       <c r="K268" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L268" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M268" t="n">
@@ -17682,7 +17682,7 @@
       </c>
       <c r="L279" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M279" t="n">
@@ -17719,7 +17719,7 @@
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G280" t="n">
@@ -17733,17 +17733,17 @@
       </c>
       <c r="J280" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_08.png</t>
+          <t>boat\boat_08.png</t>
         </is>
       </c>
       <c r="K280" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L280" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M280" t="n">
@@ -18154,7 +18154,7 @@
       </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G287" t="n">
@@ -18168,17 +18168,17 @@
       </c>
       <c r="J287" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_03.png</t>
+          <t>boat\boat_03.png</t>
         </is>
       </c>
       <c r="K287" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L287" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M287" t="n">
@@ -18422,7 +18422,7 @@
       </c>
       <c r="L291" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M291" t="n">
@@ -18528,7 +18528,7 @@
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G293" t="n">
@@ -18542,17 +18542,17 @@
       </c>
       <c r="J293" t="inlineStr">
         <is>
-          <t>broom\broom_08.png</t>
+          <t>knife\knife_08.png</t>
         </is>
       </c>
       <c r="K293" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L293" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M293" t="n">
@@ -18613,7 +18613,7 @@
       </c>
       <c r="L294" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M294" t="n">
@@ -18735,7 +18735,7 @@
       </c>
       <c r="L296" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M296" t="n">
@@ -18857,7 +18857,7 @@
       </c>
       <c r="L298" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M298" t="n">
@@ -18913,12 +18913,12 @@
       </c>
       <c r="K299" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L299" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M299" t="n">
@@ -19512,7 +19512,7 @@
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G309" t="n">
@@ -19526,17 +19526,17 @@
       </c>
       <c r="J309" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_02.png</t>
+          <t>boat\boat_02.png</t>
         </is>
       </c>
       <c r="K309" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L309" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M309" t="n">
@@ -19727,7 +19727,7 @@
       </c>
       <c r="L312" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M312" t="n">
@@ -19783,12 +19783,12 @@
       </c>
       <c r="K313" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L313" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M313" t="n">
@@ -19894,7 +19894,7 @@
       </c>
       <c r="F315" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G315" t="n">
@@ -19908,17 +19908,17 @@
       </c>
       <c r="J315" t="inlineStr">
         <is>
-          <t>broom\broom_09.png</t>
+          <t>knife\knife_09.png</t>
         </is>
       </c>
       <c r="K315" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L315" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M315" t="n">
@@ -20077,7 +20077,7 @@
       </c>
       <c r="F318" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G318" t="n">
@@ -20091,17 +20091,17 @@
       </c>
       <c r="J318" t="inlineStr">
         <is>
-          <t>broom\broom_04.png</t>
+          <t>knife\knife_04.png</t>
         </is>
       </c>
       <c r="K318" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L318" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M318" t="n">
@@ -20321,7 +20321,7 @@
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G322" t="n">
@@ -20335,7 +20335,7 @@
       </c>
       <c r="J322" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_01.png</t>
+          <t>boat\boat_01.png</t>
         </is>
       </c>
       <c r="K322" t="inlineStr">
@@ -20390,7 +20390,7 @@
       </c>
       <c r="F323" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G323" t="n">
@@ -20404,17 +20404,17 @@
       </c>
       <c r="J323" t="inlineStr">
         <is>
-          <t>broom\broom_12.png</t>
+          <t>knife\knife_12.png</t>
         </is>
       </c>
       <c r="K323" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L323" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M323" t="n">
@@ -20634,7 +20634,7 @@
       </c>
       <c r="F327" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G327" t="n">
@@ -20648,17 +20648,17 @@
       </c>
       <c r="J327" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_06.png</t>
+          <t>boat\boat_06.png</t>
         </is>
       </c>
       <c r="K327" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L327" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M327" t="n">
@@ -20719,7 +20719,7 @@
       </c>
       <c r="L328" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M328" t="n">
@@ -20817,7 +20817,7 @@
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G330" t="n">
@@ -20831,17 +20831,17 @@
       </c>
       <c r="J330" t="inlineStr">
         <is>
-          <t>broom\broom_07.png</t>
+          <t>knife\knife_07.png</t>
         </is>
       </c>
       <c r="K330" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L330" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M330" t="n">
@@ -21183,7 +21183,7 @@
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G336" t="n">
@@ -21197,17 +21197,17 @@
       </c>
       <c r="J336" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_13.png</t>
+          <t>boat\boat_13.png</t>
         </is>
       </c>
       <c r="K336" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L336" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M336" t="n">
@@ -21557,7 +21557,7 @@
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G342" t="n">
@@ -21571,17 +21571,17 @@
       </c>
       <c r="J342" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_05.png</t>
+          <t>boat\boat_05.png</t>
         </is>
       </c>
       <c r="K342" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L342" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M342" t="n">
@@ -21618,7 +21618,7 @@
       </c>
       <c r="F343" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G343" t="n">
@@ -21632,7 +21632,7 @@
       </c>
       <c r="J343" t="inlineStr">
         <is>
-          <t>broom\broom_05.png</t>
+          <t>knife\knife_05.png</t>
         </is>
       </c>
       <c r="K343" t="inlineStr">
@@ -21772,7 +21772,7 @@
       </c>
       <c r="L345" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M345" t="n">
@@ -21894,7 +21894,7 @@
       </c>
       <c r="L347" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M347" t="n">
@@ -22016,7 +22016,7 @@
       </c>
       <c r="L349" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M349" t="n">
@@ -22138,7 +22138,7 @@
       </c>
       <c r="L351" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M351" t="n">
@@ -22260,7 +22260,7 @@
       </c>
       <c r="L353" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M353" t="n">
@@ -22297,7 +22297,7 @@
       </c>
       <c r="F354" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G354" t="n">
@@ -22311,17 +22311,17 @@
       </c>
       <c r="J354" t="inlineStr">
         <is>
-          <t>broom\broom_01.png</t>
+          <t>knife\knife_01.png</t>
         </is>
       </c>
       <c r="K354" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L354" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M354" t="n">
@@ -22793,7 +22793,7 @@
       </c>
       <c r="F362" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G362" t="n">
@@ -22807,17 +22807,17 @@
       </c>
       <c r="J362" t="inlineStr">
         <is>
-          <t>broom\broom_06.png</t>
+          <t>knife\knife_06.png</t>
         </is>
       </c>
       <c r="K362" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L362" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M362" t="n">
@@ -22854,7 +22854,7 @@
       </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G363" t="n">
@@ -22868,17 +22868,17 @@
       </c>
       <c r="J363" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_11.png</t>
+          <t>boat\boat_11.png</t>
         </is>
       </c>
       <c r="K363" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L363" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M363" t="n">
@@ -23244,7 +23244,7 @@
       </c>
       <c r="L369" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M369" t="n">
@@ -23366,7 +23366,7 @@
       </c>
       <c r="L371" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M371" t="n">
@@ -23525,7 +23525,7 @@
       </c>
       <c r="F374" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G374" t="n">
@@ -23539,17 +23539,17 @@
       </c>
       <c r="J374" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_07.png</t>
+          <t>boat\boat_07.png</t>
         </is>
       </c>
       <c r="K374" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L374" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M374" t="n">
@@ -23716,7 +23716,7 @@
       </c>
       <c r="F377" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G377" t="n">
@@ -23730,17 +23730,17 @@
       </c>
       <c r="J377" t="inlineStr">
         <is>
-          <t>broom\broom_02.png</t>
+          <t>knife\knife_02.png</t>
         </is>
       </c>
       <c r="K377" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L377" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M377" t="n">
@@ -23907,7 +23907,7 @@
       </c>
       <c r="F380" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G380" t="n">
@@ -23921,17 +23921,17 @@
       </c>
       <c r="J380" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_10.png</t>
+          <t>boat\boat_10.png</t>
         </is>
       </c>
       <c r="K380" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L380" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M380" t="n">
@@ -24029,7 +24029,7 @@
       </c>
       <c r="F382" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G382" t="n">
@@ -24043,17 +24043,17 @@
       </c>
       <c r="J382" t="inlineStr">
         <is>
-          <t>broom\broom_11.png</t>
+          <t>knife\knife_11.png</t>
         </is>
       </c>
       <c r="K382" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L382" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M382" t="n">
@@ -24212,7 +24212,7 @@
       </c>
       <c r="F385" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G385" t="n">
@@ -24226,17 +24226,17 @@
       </c>
       <c r="J385" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_03.png</t>
+          <t>boat\boat_03.png</t>
         </is>
       </c>
       <c r="K385" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L385" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M385" t="n">
@@ -24456,7 +24456,7 @@
       </c>
       <c r="F389" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G389" t="n">
@@ -24470,17 +24470,17 @@
       </c>
       <c r="J389" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_06.png</t>
+          <t>boat\boat_06.png</t>
         </is>
       </c>
       <c r="K389" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L389" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M389" t="n">
@@ -24536,12 +24536,12 @@
       </c>
       <c r="K390" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L390" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M390" t="n">
@@ -24854,7 +24854,7 @@
       </c>
       <c r="L395" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M395" t="n">
@@ -25318,7 +25318,7 @@
       </c>
       <c r="F403" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G403" t="n">
@@ -25332,17 +25332,17 @@
       </c>
       <c r="J403" t="inlineStr">
         <is>
-          <t>broom\broom_01.png</t>
+          <t>knife\knife_01.png</t>
         </is>
       </c>
       <c r="K403" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L403" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M403" t="n">
@@ -25403,7 +25403,7 @@
       </c>
       <c r="L404" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M404" t="n">
@@ -25562,7 +25562,7 @@
       </c>
       <c r="F407" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G407" t="n">
@@ -25576,17 +25576,17 @@
       </c>
       <c r="J407" t="inlineStr">
         <is>
-          <t>broom\broom_08.png</t>
+          <t>knife\knife_08.png</t>
         </is>
       </c>
       <c r="K407" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L407" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M407" t="n">
@@ -25745,7 +25745,7 @@
       </c>
       <c r="F410" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G410" t="n">
@@ -25759,7 +25759,7 @@
       </c>
       <c r="J410" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_04.png</t>
+          <t>boat\boat_04.png</t>
         </is>
       </c>
       <c r="K410" t="inlineStr">
@@ -25875,7 +25875,7 @@
       </c>
       <c r="F412" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G412" t="n">
@@ -25889,17 +25889,17 @@
       </c>
       <c r="J412" t="inlineStr">
         <is>
-          <t>broom\broom_11.png</t>
+          <t>knife\knife_11.png</t>
         </is>
       </c>
       <c r="K412" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L412" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M412" t="n">
@@ -25936,7 +25936,7 @@
       </c>
       <c r="F413" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G413" t="n">
@@ -25950,17 +25950,17 @@
       </c>
       <c r="J413" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_05.png</t>
+          <t>boat\boat_05.png</t>
         </is>
       </c>
       <c r="K413" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L413" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M413" t="n">
@@ -26119,7 +26119,7 @@
       </c>
       <c r="F416" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G416" t="n">
@@ -26133,17 +26133,17 @@
       </c>
       <c r="J416" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_11.png</t>
+          <t>boat\boat_11.png</t>
         </is>
       </c>
       <c r="K416" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L416" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M416" t="n">
@@ -26265,7 +26265,7 @@
       </c>
       <c r="L418" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M418" t="n">
@@ -26668,7 +26668,7 @@
       </c>
       <c r="F425" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G425" t="n">
@@ -26682,7 +26682,7 @@
       </c>
       <c r="J425" t="inlineStr">
         <is>
-          <t>broom\broom_12.png</t>
+          <t>knife\knife_12.png</t>
         </is>
       </c>
       <c r="K425" t="inlineStr">
@@ -26944,7 +26944,7 @@
       </c>
       <c r="L429" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M429" t="n">
@@ -27371,7 +27371,7 @@
       </c>
       <c r="L436" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M436" t="n">
@@ -27408,7 +27408,7 @@
       </c>
       <c r="F437" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G437" t="n">
@@ -27422,17 +27422,17 @@
       </c>
       <c r="J437" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_03.png</t>
+          <t>boat\boat_03.png</t>
         </is>
       </c>
       <c r="K437" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L437" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M437" t="n">
@@ -27652,7 +27652,7 @@
       </c>
       <c r="F441" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G441" t="n">
@@ -27666,17 +27666,17 @@
       </c>
       <c r="J441" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_08.png</t>
+          <t>boat\boat_08.png</t>
         </is>
       </c>
       <c r="K441" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L441" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M441" t="n">
@@ -27737,7 +27737,7 @@
       </c>
       <c r="L442" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M442" t="n">
@@ -27923,12 +27923,12 @@
       </c>
       <c r="K445" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L445" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M445" t="n">
@@ -28119,7 +28119,7 @@
       </c>
       <c r="L448" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M448" t="n">
@@ -28339,7 +28339,7 @@
       </c>
       <c r="F452" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G452" t="n">
@@ -28353,17 +28353,17 @@
       </c>
       <c r="J452" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_01.png</t>
+          <t>boat\boat_01.png</t>
         </is>
       </c>
       <c r="K452" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L452" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M452" t="n">
@@ -28729,7 +28729,7 @@
       </c>
       <c r="L458" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M458" t="n">
@@ -28896,7 +28896,7 @@
       </c>
       <c r="F461" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G461" t="n">
@@ -28910,17 +28910,17 @@
       </c>
       <c r="J461" t="inlineStr">
         <is>
-          <t>broom\broom_04.png</t>
+          <t>knife\knife_04.png</t>
         </is>
       </c>
       <c r="K461" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L461" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M461" t="n">
@@ -29018,7 +29018,7 @@
       </c>
       <c r="F463" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G463" t="n">
@@ -29032,17 +29032,17 @@
       </c>
       <c r="J463" t="inlineStr">
         <is>
-          <t>broom\broom_09.png</t>
+          <t>knife\knife_09.png</t>
         </is>
       </c>
       <c r="K463" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L463" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M463" t="n">
@@ -29164,7 +29164,7 @@
       </c>
       <c r="L465" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M465" t="n">
@@ -29201,7 +29201,7 @@
       </c>
       <c r="F466" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G466" t="n">
@@ -29215,17 +29215,17 @@
       </c>
       <c r="J466" t="inlineStr">
         <is>
-          <t>broom\broom_10.png</t>
+          <t>knife\knife_10.png</t>
         </is>
       </c>
       <c r="K466" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L466" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M466" t="n">
@@ -29464,12 +29464,12 @@
       </c>
       <c r="K470" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L470" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M470" t="n">
@@ -29843,7 +29843,7 @@
       </c>
       <c r="L476" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M476" t="n">
@@ -30620,7 +30620,7 @@
       </c>
       <c r="F489" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G489" t="n">
@@ -30634,17 +30634,17 @@
       </c>
       <c r="J489" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_12.png</t>
+          <t>boat\boat_12.png</t>
         </is>
       </c>
       <c r="K489" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L489" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M489" t="n">
@@ -30742,7 +30742,7 @@
       </c>
       <c r="F491" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G491" t="n">
@@ -30756,17 +30756,17 @@
       </c>
       <c r="J491" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_13.png</t>
+          <t>boat\boat_13.png</t>
         </is>
       </c>
       <c r="K491" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L491" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M491" t="n">
@@ -30864,7 +30864,7 @@
       </c>
       <c r="F493" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G493" t="n">
@@ -30878,17 +30878,17 @@
       </c>
       <c r="J493" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_02.png</t>
+          <t>boat\boat_02.png</t>
         </is>
       </c>
       <c r="K493" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L493" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M493" t="n">
@@ -30949,7 +30949,7 @@
       </c>
       <c r="L494" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M494" t="n">
@@ -30986,7 +30986,7 @@
       </c>
       <c r="F495" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G495" t="n">
@@ -31000,17 +31000,17 @@
       </c>
       <c r="J495" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_07.png</t>
+          <t>boat\boat_07.png</t>
         </is>
       </c>
       <c r="K495" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L495" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M495" t="n">
@@ -31047,7 +31047,7 @@
       </c>
       <c r="F496" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G496" t="n">
@@ -31061,7 +31061,7 @@
       </c>
       <c r="J496" t="inlineStr">
         <is>
-          <t>broom\broom_03.png</t>
+          <t>knife\knife_03.png</t>
         </is>
       </c>
       <c r="K496" t="inlineStr">
@@ -31071,7 +31071,7 @@
       </c>
       <c r="L496" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M496" t="n">
@@ -31201,7 +31201,7 @@
       </c>
       <c r="L498" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M498" t="n">
@@ -31323,7 +31323,7 @@
       </c>
       <c r="L500" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M500" t="n">
@@ -31421,7 +31421,7 @@
       </c>
       <c r="F502" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G502" t="n">
@@ -31435,17 +31435,17 @@
       </c>
       <c r="J502" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_09.png</t>
+          <t>boat\boat_09.png</t>
         </is>
       </c>
       <c r="K502" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L502" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M502" t="n">
@@ -31551,7 +31551,7 @@
       </c>
       <c r="F504" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G504" t="n">
@@ -31565,17 +31565,17 @@
       </c>
       <c r="J504" t="inlineStr">
         <is>
-          <t>broom\broom_07.png</t>
+          <t>knife\knife_07.png</t>
         </is>
       </c>
       <c r="K504" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L504" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M504" t="n">
@@ -31673,7 +31673,7 @@
       </c>
       <c r="F506" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G506" t="n">
@@ -31687,17 +31687,17 @@
       </c>
       <c r="J506" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_04.png</t>
+          <t>boat\boat_04.png</t>
         </is>
       </c>
       <c r="K506" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L506" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M506" t="n">
@@ -31819,7 +31819,7 @@
       </c>
       <c r="L508" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M508" t="n">
@@ -31978,7 +31978,7 @@
       </c>
       <c r="F511" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G511" t="n">
@@ -31992,17 +31992,17 @@
       </c>
       <c r="J511" t="inlineStr">
         <is>
-          <t>broom\broom_06.png</t>
+          <t>knife\knife_06.png</t>
         </is>
       </c>
       <c r="K511" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L511" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M511" t="n">
@@ -32222,7 +32222,7 @@
       </c>
       <c r="F515" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G515" t="n">
@@ -32236,17 +32236,17 @@
       </c>
       <c r="J515" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_10.png</t>
+          <t>boat\boat_10.png</t>
         </is>
       </c>
       <c r="K515" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L515" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M515" t="n">
@@ -32498,7 +32498,7 @@
       </c>
       <c r="L519" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M519" t="n">
@@ -32535,7 +32535,7 @@
       </c>
       <c r="F520" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G520" t="n">
@@ -32549,17 +32549,17 @@
       </c>
       <c r="J520" t="inlineStr">
         <is>
-          <t>broom\broom_09.png</t>
+          <t>knife\knife_09.png</t>
         </is>
       </c>
       <c r="K520" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L520" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M520" t="n">
@@ -32901,7 +32901,7 @@
       </c>
       <c r="F526" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G526" t="n">
@@ -32915,17 +32915,17 @@
       </c>
       <c r="J526" t="inlineStr">
         <is>
-          <t>broom\broom_02.png</t>
+          <t>knife\knife_02.png</t>
         </is>
       </c>
       <c r="K526" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L526" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M526" t="n">
@@ -32962,7 +32962,7 @@
       </c>
       <c r="F527" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G527" t="n">
@@ -32976,17 +32976,17 @@
       </c>
       <c r="J527" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_11.png</t>
+          <t>boat\boat_11.png</t>
         </is>
       </c>
       <c r="K527" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L527" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M527" t="n">
@@ -33145,7 +33145,7 @@
       </c>
       <c r="F530" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G530" t="n">
@@ -33159,17 +33159,17 @@
       </c>
       <c r="J530" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_06.png</t>
+          <t>boat\boat_06.png</t>
         </is>
       </c>
       <c r="K530" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L530" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M530" t="n">
@@ -33763,7 +33763,7 @@
       </c>
       <c r="F540" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G540" t="n">
@@ -33777,17 +33777,17 @@
       </c>
       <c r="J540" t="inlineStr">
         <is>
-          <t>broom\broom_05.png</t>
+          <t>knife\knife_05.png</t>
         </is>
       </c>
       <c r="K540" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L540" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M540" t="n">
@@ -34092,7 +34092,7 @@
       </c>
       <c r="L545" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M545" t="n">
@@ -34209,12 +34209,12 @@
       </c>
       <c r="K547" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L547" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M547" t="n">
@@ -34283,7 +34283,7 @@
       </c>
       <c r="L548" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M548" t="n">
@@ -34405,7 +34405,7 @@
       </c>
       <c r="L550" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M550" t="n">
@@ -34747,7 +34747,7 @@
       </c>
       <c r="F556" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G556" t="n">
@@ -34761,17 +34761,17 @@
       </c>
       <c r="J556" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_12.png</t>
+          <t>boat\boat_12.png</t>
         </is>
       </c>
       <c r="K556" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L556" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M556" t="n">
@@ -34869,7 +34869,7 @@
       </c>
       <c r="F558" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G558" t="n">
@@ -34883,17 +34883,17 @@
       </c>
       <c r="J558" t="inlineStr">
         <is>
-          <t>broom\broom_04.png</t>
+          <t>knife\knife_04.png</t>
         </is>
       </c>
       <c r="K558" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L558" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M558" t="n">
@@ -35052,7 +35052,7 @@
       </c>
       <c r="F561" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G561" t="n">
@@ -35066,17 +35066,17 @@
       </c>
       <c r="J561" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_03.png</t>
+          <t>boat\boat_03.png</t>
         </is>
       </c>
       <c r="K561" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L561" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M561" t="n">
@@ -35450,7 +35450,7 @@
       </c>
       <c r="L567" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M567" t="n">
@@ -35617,7 +35617,7 @@
       </c>
       <c r="F570" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G570" t="n">
@@ -35631,17 +35631,17 @@
       </c>
       <c r="J570" t="inlineStr">
         <is>
-          <t>broom\broom_05.png</t>
+          <t>knife\knife_05.png</t>
         </is>
       </c>
       <c r="K570" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L570" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M570" t="n">
@@ -35861,7 +35861,7 @@
       </c>
       <c r="F574" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G574" t="n">
@@ -35875,17 +35875,17 @@
       </c>
       <c r="J574" t="inlineStr">
         <is>
-          <t>broom\broom_07.png</t>
+          <t>knife\knife_07.png</t>
         </is>
       </c>
       <c r="K574" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L574" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M574" t="n">
@@ -35946,7 +35946,7 @@
       </c>
       <c r="L575" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M575" t="n">
@@ -36312,7 +36312,7 @@
       </c>
       <c r="L581" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M581" t="n">
@@ -36471,7 +36471,7 @@
       </c>
       <c r="F584" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G584" t="n">
@@ -36485,17 +36485,17 @@
       </c>
       <c r="J584" t="inlineStr">
         <is>
-          <t>broom\broom_02.png</t>
+          <t>knife\knife_02.png</t>
         </is>
       </c>
       <c r="K584" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L584" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M584" t="n">
@@ -36662,7 +36662,7 @@
       </c>
       <c r="F587" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G587" t="n">
@@ -36676,17 +36676,17 @@
       </c>
       <c r="J587" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_07.png</t>
+          <t>boat\boat_07.png</t>
         </is>
       </c>
       <c r="K587" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L587" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M587" t="n">
@@ -36991,7 +36991,7 @@
       </c>
       <c r="L592" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M592" t="n">
@@ -37028,7 +37028,7 @@
       </c>
       <c r="F593" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G593" t="n">
@@ -37042,17 +37042,17 @@
       </c>
       <c r="J593" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_09.png</t>
+          <t>boat\boat_09.png</t>
         </is>
       </c>
       <c r="K593" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L593" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M593" t="n">
@@ -37150,7 +37150,7 @@
       </c>
       <c r="F595" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G595" t="n">
@@ -37164,17 +37164,17 @@
       </c>
       <c r="J595" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_13.png</t>
+          <t>boat\boat_13.png</t>
         </is>
       </c>
       <c r="K595" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L595" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M595" t="n">
@@ -37333,7 +37333,7 @@
       </c>
       <c r="F598" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G598" t="n">
@@ -37347,7 +37347,7 @@
       </c>
       <c r="J598" t="inlineStr">
         <is>
-          <t>broom\broom_11.png</t>
+          <t>knife\knife_11.png</t>
         </is>
       </c>
       <c r="K598" t="inlineStr">
@@ -37487,7 +37487,7 @@
       </c>
       <c r="L600" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M600" t="n">
@@ -37890,7 +37890,7 @@
       </c>
       <c r="F607" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G607" t="n">
@@ -37904,17 +37904,17 @@
       </c>
       <c r="J607" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_10.png</t>
+          <t>boat\boat_10.png</t>
         </is>
       </c>
       <c r="K607" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L607" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M607" t="n">
@@ -37951,7 +37951,7 @@
       </c>
       <c r="F608" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G608" t="n">
@@ -37965,17 +37965,17 @@
       </c>
       <c r="J608" t="inlineStr">
         <is>
-          <t>broom\broom_08.png</t>
+          <t>knife\knife_08.png</t>
         </is>
       </c>
       <c r="K608" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L608" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M608" t="n">
@@ -38158,7 +38158,7 @@
       </c>
       <c r="L611" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M611" t="n">
@@ -38288,7 +38288,7 @@
       </c>
       <c r="L613" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M613" t="n">
@@ -38516,7 +38516,7 @@
       </c>
       <c r="F617" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G617" t="n">
@@ -38530,17 +38530,17 @@
       </c>
       <c r="J617" t="inlineStr">
         <is>
-          <t>broom\broom_12.png</t>
+          <t>knife\knife_12.png</t>
         </is>
       </c>
       <c r="K617" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L617" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M617" t="n">
@@ -38638,7 +38638,7 @@
       </c>
       <c r="F619" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G619" t="n">
@@ -38652,17 +38652,17 @@
       </c>
       <c r="J619" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_08.png</t>
+          <t>boat\boat_08.png</t>
         </is>
       </c>
       <c r="K619" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L619" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M619" t="n">
@@ -38699,7 +38699,7 @@
       </c>
       <c r="F620" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G620" t="n">
@@ -38713,17 +38713,17 @@
       </c>
       <c r="J620" t="inlineStr">
         <is>
-          <t>broom\broom_06.png</t>
+          <t>knife\knife_06.png</t>
         </is>
       </c>
       <c r="K620" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L620" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M620" t="n">
@@ -38821,7 +38821,7 @@
       </c>
       <c r="F622" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G622" t="n">
@@ -38835,17 +38835,17 @@
       </c>
       <c r="J622" t="inlineStr">
         <is>
-          <t>broom\broom_10.png</t>
+          <t>knife\knife_10.png</t>
         </is>
       </c>
       <c r="K622" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L622" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M622" t="n">
@@ -38943,7 +38943,7 @@
       </c>
       <c r="F624" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G624" t="n">
@@ -38957,7 +38957,7 @@
       </c>
       <c r="J624" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_02.png</t>
+          <t>boat\boat_02.png</t>
         </is>
       </c>
       <c r="K624" t="inlineStr">
@@ -39805,7 +39805,7 @@
       </c>
       <c r="F638" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G638" t="n">
@@ -39819,17 +39819,17 @@
       </c>
       <c r="J638" t="inlineStr">
         <is>
-          <t>broom\broom_03.png</t>
+          <t>knife\knife_03.png</t>
         </is>
       </c>
       <c r="K638" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L638" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M638" t="n">
@@ -39866,7 +39866,7 @@
       </c>
       <c r="F639" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G639" t="n">
@@ -39880,17 +39880,17 @@
       </c>
       <c r="J639" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_01.png</t>
+          <t>boat\boat_01.png</t>
         </is>
       </c>
       <c r="K639" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L639" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M639" t="n">
@@ -40012,7 +40012,7 @@
       </c>
       <c r="L641" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M641" t="n">
@@ -40110,7 +40110,7 @@
       </c>
       <c r="F643" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="G643" t="n">
@@ -40124,17 +40124,17 @@
       </c>
       <c r="J643" t="inlineStr">
         <is>
-          <t>sailboat\sailboat_05.png</t>
+          <t>boat\boat_05.png</t>
         </is>
       </c>
       <c r="K643" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L643" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M643" t="n">
@@ -40293,7 +40293,7 @@
       </c>
       <c r="F646" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="G646" t="n">
@@ -40307,17 +40307,17 @@
       </c>
       <c r="J646" t="inlineStr">
         <is>
-          <t>broom\broom_01.png</t>
+          <t>knife\knife_01.png</t>
         </is>
       </c>
       <c r="K646" t="inlineStr">
         <is>
-          <t>broom</t>
+          <t>knife</t>
         </is>
       </c>
       <c r="L646" t="inlineStr">
         <is>
-          <t>Besen</t>
+          <t>Messer</t>
         </is>
       </c>
       <c r="M646" t="n">
@@ -40378,7 +40378,7 @@
       </c>
       <c r="L647" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M647" t="n">
@@ -40691,7 +40691,7 @@
       </c>
       <c r="L652" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M652" t="n">
@@ -40808,12 +40808,12 @@
       </c>
       <c r="K654" t="inlineStr">
         <is>
-          <t>sailboat</t>
+          <t>boat</t>
         </is>
       </c>
       <c r="L654" t="inlineStr">
         <is>
-          <t>Segelboot</t>
+          <t>Boot</t>
         </is>
       </c>
       <c r="M654" t="n">
@@ -40943,7 +40943,7 @@
       </c>
       <c r="L656" t="inlineStr">
         <is>
-          <t>Stecknadel</t>
+          <t>Nadel</t>
         </is>
       </c>
       <c r="M656" t="n">

</xml_diff>